<commit_message>
chore: run 2026-03-17 14:18 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_17_03_2026.xlsx
+++ b/logs/Consolidado_17_03_2026.xlsx
@@ -638,10 +638,10 @@
         <v>156</v>
       </c>
       <c r="C2" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
@@ -657,10 +657,10 @@
         <v>66</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -676,10 +676,10 @@
         <v>79</v>
       </c>
       <c r="C4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -695,10 +695,10 @@
         <v>71</v>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -714,10 +714,10 @@
         <v>47</v>
       </c>
       <c r="C6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -733,10 +733,10 @@
         <v>106</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>4</v>
@@ -752,10 +752,10 @@
         <v>9</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>10</v>
@@ -1068,80 +1068,80 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Antirougeurs Rosamed SPF50+
 Concentrado Hidratante Pele Tendência Vermelhidão
 30 ml</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/antirougeurs-rosamed-spf50-8429965.html</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>8429965</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Body 24H Deodorant Soothing No Alcohol
 Desodorizante Roll-On 24H Pele Sensível
 50 ml</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/body-24h-deodorant-soothing-no-alcohol-6938680.html</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>6938680</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -1267,40 +1267,40 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Cicalfate+ Absorbing Repair Spray
 Spray Secante e Reparador Zonas Irritadas
 100ml</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cicalfate-absorbing-repair-spray-7268424.html</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>7268424</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -1347,40 +1347,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Cicalfate+ Hydrating Skin Repairing Emulsion
 Creme Hidratante Pós-Cirúrgico e Pós-Tatuagem
 40 ml</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cicalfate-hydrating-skin-repairing-emulsion-7632459.html</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>7632459</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -1466,80 +1466,80 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Cicalfate+ Purifying Cleansing Gel
 Gel de Limpeza Purificante da Pele Irritada
 200 ml</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cicalfate-purifying-cleansing-gel-7632460.html</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>7632460</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Cicalfate+ Repair Lip Blam
 Bálsamo Repara e Protege Lábios Gretados 24H
 12 ml</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cicalfate-repair-lip-blam-7850120.html</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>7850120</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -1632,40 +1632,40 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Cicalfate+ Scar Gel
 Gel Reduz e Melhora Aspeto das Cicatrizes
 40 ml</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cicalfate-scar-gel-8726970.html</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>8726970</t>
         </is>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -1958,40 +1958,40 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Cleanance Comedomed Peeling Cleansing Gel
 Gel de Limpeza esfoliante pele com Acne
 400 ml</t>
         </is>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cleanance-comedomed-peeling-cleansing-gel-8660052.html</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>8660052</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -2723,40 +2723,40 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Couvrance Fluid Foundation Corrector 4.0
 Base Fluída Corretora SPF20
 30 ml</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/couvrance-fluid-foundation-corrector-4.0-3599500.html</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr"/>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>3599500</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -2803,40 +2803,40 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Couvrance High Definition Mascara Black
 Máscara de Pestanas Alta Definição Preta
 7 ml</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/couvrance-high-definition-mascara-black-8154716.html</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr"/>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>8154716</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H51" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -2963,80 +2963,80 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Dermabsolu Concentrated Resculpting Serum
 Sérum Anti Idade Rugas e Firmeza
 30 ml</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermabsolu-concentrated-resculpting-serum-6739621.html</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>6739621</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>Dermabsolu Eco-Refill Redensifying Day Cream
 Recarga Creme anti idade Rugas e Firmeza
 50 ml</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/dermabsolu-eco-refill-redensifying-day-cream-8152747.html</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr"/>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr"/>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
         <is>
           <t>8152747</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="H56" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -3083,40 +3083,40 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B58" s="7" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Dermabsolu Intensive Resculpting Night Cream
 Creme Noite Anti Idade Rugas e Firmeza
 40 ml</t>
         </is>
       </c>
-      <c r="D58" s="7" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/dermabsolu-intensive-resculpting-night-cream-8152748.html</t>
         </is>
       </c>
-      <c r="E58" s="7" t="inlineStr"/>
-      <c r="F58" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>8152748</t>
         </is>
       </c>
-      <c r="H58" s="7" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -3323,40 +3323,40 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Hyaluron Activ B3 Cell Renewal Aqua Cream-Gel
 Creme-Gel Dia Rugas AH, Niacinamida
 50 ml</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/hyaluron-activ-b3-cell-renewal-aqua-cream-gel-7982205.html</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr"/>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>7982205</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -3603,40 +3603,40 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C71" s="5" t="inlineStr">
         <is>
           <t>Hyaluron Activ B3 Triple Correction Eye Cream
 Creme de Olhos Rugas Olheiras Papos
 15 ml</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/hyaluron-activ-b3-triple-correction-eye-cream-7654174.html</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr"/>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="E71" s="5" t="inlineStr"/>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>7654174</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -4283,40 +4283,40 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B88" s="7" t="inlineStr">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C88" s="7" t="inlineStr">
+      <c r="C88" s="3" t="inlineStr">
         <is>
           <t>MEN Shaving Foam
 Espuma de Barbear Calmante sem Álcool
 200ml</t>
         </is>
       </c>
-      <c r="D88" s="7" t="inlineStr">
+      <c r="D88" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/men-shaving-foam-3000655.html</t>
         </is>
       </c>
-      <c r="E88" s="7" t="inlineStr"/>
-      <c r="F88" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G88" s="7" t="inlineStr">
+      <c r="E88" s="3" t="inlineStr"/>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
         <is>
           <t>3000655</t>
         </is>
       </c>
-      <c r="H88" s="7" t="inlineStr">
+      <c r="H88" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -4449,40 +4449,40 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B92" s="7" t="inlineStr">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C92" s="7" t="inlineStr">
+      <c r="C92" s="5" t="inlineStr">
         <is>
           <t>Milk Cleanser Dry Sensitive Skin
 Leite de Limpeza Desmaquilhante Pele Seca
 200 ml</t>
         </is>
       </c>
-      <c r="D92" s="7" t="inlineStr">
+      <c r="D92" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/milk-cleanser-dry-sensitive-skin-3001085.html</t>
         </is>
       </c>
-      <c r="E92" s="7" t="inlineStr"/>
-      <c r="F92" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="inlineStr">
+      <c r="E92" s="5" t="inlineStr"/>
+      <c r="F92" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
         <is>
           <t>3001085</t>
         </is>
       </c>
-      <c r="H92" s="7" t="inlineStr">
+      <c r="H92" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -6342,40 +6342,40 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B139" s="7" t="inlineStr">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C139" s="7" t="inlineStr">
+      <c r="C139" s="5" t="inlineStr">
         <is>
           <t>Tolérance Extremely Gentle Cleanser
 Gel de Limpeza Pele Reativa e Intolerante
 200 ml</t>
         </is>
       </c>
-      <c r="D139" s="7" t="inlineStr">
+      <c r="D139" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/tolerance-extremely-gentle-cleanser-7378122.html</t>
         </is>
       </c>
-      <c r="E139" s="7" t="inlineStr"/>
-      <c r="F139" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G139" s="7" t="inlineStr">
+      <c r="E139" s="5" t="inlineStr"/>
+      <c r="F139" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="inlineStr">
         <is>
           <t>7378122</t>
         </is>
       </c>
-      <c r="H139" s="7" t="inlineStr">
+      <c r="H139" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -6788,40 +6788,40 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B150" s="7" t="inlineStr">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C150" s="7" t="inlineStr">
+      <c r="C150" s="5" t="inlineStr">
         <is>
           <t>Vitamin Activ Cg Eco-Refill Radiance Cream
 Recarga Creme Rugas Vitamina C
 50 ml</t>
         </is>
       </c>
-      <c r="D150" s="7" t="inlineStr">
+      <c r="D150" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/vitamin-activ-cg-eco-refill-radiance-cream-7982202.html</t>
         </is>
       </c>
-      <c r="E150" s="7" t="inlineStr"/>
-      <c r="F150" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G150" s="7" t="inlineStr">
+      <c r="E150" s="5" t="inlineStr"/>
+      <c r="F150" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G150" s="5" t="inlineStr">
         <is>
           <t>7982202</t>
         </is>
       </c>
-      <c r="H150" s="7" t="inlineStr">
+      <c r="H150" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -6948,40 +6948,40 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B154" s="7" t="inlineStr">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C154" s="7" t="inlineStr">
+      <c r="C154" s="5" t="inlineStr">
         <is>
           <t>Xeracalm A.D Lipid-Replenishing Balm
 Bálsamo Relipidante Pele Seca Atópica Comichão
 200 ml</t>
         </is>
       </c>
-      <c r="D154" s="7" t="inlineStr">
+      <c r="D154" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/xeracalm-a.d-lipid-replenishing-balm-5195068.html</t>
         </is>
       </c>
-      <c r="E154" s="7" t="inlineStr"/>
-      <c r="F154" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G154" s="7" t="inlineStr">
+      <c r="E154" s="5" t="inlineStr"/>
+      <c r="F154" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G154" s="5" t="inlineStr">
         <is>
           <t>5195068</t>
         </is>
       </c>
-      <c r="H154" s="7" t="inlineStr">
+      <c r="H154" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -7068,40 +7068,40 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B157" s="7" t="inlineStr">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C157" s="7" t="inlineStr">
+      <c r="C157" s="3" t="inlineStr">
         <is>
           <t>Xeracalm A.D Lipid-Replenishing Cleansing Oil
 Óleo de Limpeza Pele Seca Atópica Comichão
 750 ml</t>
         </is>
       </c>
-      <c r="D157" s="7" t="inlineStr">
+      <c r="D157" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/xeracalm-a.d-lipid-replenishing-cleansing-oil-7889347.html</t>
         </is>
       </c>
-      <c r="E157" s="7" t="inlineStr"/>
-      <c r="F157" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G157" s="7" t="inlineStr">
+      <c r="E157" s="3" t="inlineStr"/>
+      <c r="F157" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="inlineStr">
         <is>
           <t>7889347</t>
         </is>
       </c>
-      <c r="H157" s="7" t="inlineStr">
+      <c r="H157" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -7188,40 +7188,40 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B160" s="7" t="inlineStr">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C160" s="7" t="inlineStr">
+      <c r="C160" s="5" t="inlineStr">
         <is>
           <t>Xeracalm A.D Soothing Concentrate
 Creme Concentrado SOS Pele Atópica Comichão
 40 ml</t>
         </is>
       </c>
-      <c r="D160" s="7" t="inlineStr">
+      <c r="D160" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/xeracalm-a.d-soothing-concentrate-8487592.html</t>
         </is>
       </c>
-      <c r="E160" s="7" t="inlineStr"/>
-      <c r="F160" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G160" s="7" t="inlineStr">
+      <c r="E160" s="5" t="inlineStr"/>
+      <c r="F160" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G160" s="5" t="inlineStr">
         <is>
           <t>8487592</t>
         </is>
       </c>
-      <c r="H160" s="7" t="inlineStr">
+      <c r="H160" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -7388,40 +7388,40 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B165" s="7" t="inlineStr">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C165" s="7" t="inlineStr">
+      <c r="C165" s="3" t="inlineStr">
         <is>
           <t>Xeracalm NUTRITION Moisturizing Lotion
 Leite Hidratante Pele Seca Secagem Rápida
 400 ml</t>
         </is>
       </c>
-      <c r="D165" s="7" t="inlineStr">
+      <c r="D165" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/xeracalm-nutrition-moisturizing-lotion-443918.html</t>
         </is>
       </c>
-      <c r="E165" s="7" t="inlineStr"/>
-      <c r="F165" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G165" s="7" t="inlineStr">
+      <c r="E165" s="3" t="inlineStr"/>
+      <c r="F165" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="inlineStr">
         <is>
           <t>7816801</t>
         </is>
       </c>
-      <c r="H165" s="7" t="inlineStr">
+      <c r="H165" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -7983,40 +7983,40 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Creme Palpebral Eczema Dexyane Med
 Creme Eczema da Pálpebra
 15 ml</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/creme-palpebral-eczema-dexyane-med-7024952.html</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>7024952</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -8915,40 +8915,40 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Kelual Squanorm Anti-Dandruff Refreshing
 Champô Resfrescante Cabelo com Caspa
 200 ml</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/kelual-squanorm-anti-dandruff-refreshing-8710845.html</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr"/>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>8710845</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H36" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -9129,40 +9129,40 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Keracnyl Anti-blemishes Regulating Serum
 Sérum Anti-Imperfeições Sebo-Regulador Acne
 30 ml</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/keracnyl-anti-blemishes-regulating-serum-8539819.html</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr"/>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
         <is>
           <t>8539819</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -9849,40 +9849,40 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B59" s="7" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>Ducray</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Melascreen Fluide Antitaches Brunes
 Fluido de Rosto Antimanchas Pele Mista SPF50+
 50 ml</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/melascreen-fluide-antitaches-brunes-7850427.html</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr"/>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
         <is>
           <t>7850427</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -10964,83 +10964,83 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Conditioner
 Condicionador Camomila Brilho Cabelo Loiro
 200 ml</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-conditioner-5870419.html</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>5870419</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Shampoo
 Champô Camomila Reflexos Dourado Cabelo Loiro</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-shampoo-343981.html</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>3000697</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -11610,40 +11610,40 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Cupuaçu Repairing CICA-shampoo
 Champô Cupuaçu Nutre Repara Cabelo Muito Seco
 200 ml</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-repairing-cica-shampoo-8500174.html</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>8500174</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -12541,43 +12541,43 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C52" s="7" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Manga Nourishing Conditioner
 Condicionador Manga Nutritivo Cabelo Seco</t>
         </is>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/manga-nourishing-conditioner-343975.html</t>
         </is>
       </c>
-      <c r="E52" s="7" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
         <is>
           <t>6128332</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -13042,43 +13042,43 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B64" s="7" t="inlineStr">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Nettle Oil Control Shampoo
 Champô Ortiga BIO Purifica Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="D64" s="7" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-oil-control-shampoo-343980.html</t>
         </is>
       </c>
-      <c r="E64" s="7" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G64" s="7" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
         <is>
           <t>3688262</t>
         </is>
       </c>
-      <c r="H64" s="7" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
@@ -13340,43 +13340,43 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B71" s="7" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
 Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
         </is>
       </c>
-      <c r="D71" s="7" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
         </is>
       </c>
-      <c r="E71" s="7" t="inlineStr">
+      <c r="E71" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
         <is>
           <t>7831154</t>
         </is>
       </c>
-      <c r="H71" s="7" t="inlineStr">
+      <c r="H71" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -14247,40 +14247,40 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B93" s="7" t="inlineStr">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
         <is>
           <t>Tamanu &amp; Monoi Nutri-Repair Sun Shampoo
 Champô Protetor Solar Cabelo Exposto ao Sol
 200 ml</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/tamanu-and-monoi-nutri-repair-sun-shampoo-7396246.html</t>
         </is>
       </c>
-      <c r="E93" s="7" t="inlineStr"/>
-      <c r="F93" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="inlineStr">
+      <c r="E93" s="5" t="inlineStr"/>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
         <is>
           <t>7396246</t>
         </is>
       </c>
-      <c r="H93" s="7" t="inlineStr">
+      <c r="H93" s="5" t="inlineStr">
         <is>
           <t>37%</t>
         </is>
@@ -14635,40 +14635,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Absolue Kératine Renewal Care Serum
 Sérum Reparador Extremo Pontas Danificadas
 30 ml</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/absolue-keratine-renewal-care-serum-7447296.html</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>7447296</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -15401,39 +15401,39 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Laca Sytle
 100 ml</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/laca-sytle-7447298.html</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>7447298</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>29%</t>
         </is>
@@ -15888,40 +15888,40 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Okara Blond Brightening Spray Blond Hair
 Spray Cabelo Iluminador Louro Natural ou Pintado
 150 ml</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/okara-blond-brightening-spray-blond-hair-6761000.html</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr"/>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>6761000</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -16208,40 +16208,40 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Style Holding Spray Precise &amp; Strong
 Spray Cabelo Fixação Ultra-Forte Longa Duração
 150 ml</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/style-holding-spray-precise-and-strong-7447299.html</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>7447299</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -17342,80 +17342,80 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="C73" s="3" t="inlineStr">
         <is>
           <t>Triphasic Texturizing Detangling Conditioner
 Condicionador Queda de Cabelo Texturarizante
 150 ml</t>
         </is>
       </c>
-      <c r="D73" s="7" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-texturizing-detangling-conditioner-6856570.html</t>
         </is>
       </c>
-      <c r="E73" s="7" t="inlineStr"/>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="inlineStr">
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
         <is>
           <t>6856570</t>
         </is>
       </c>
-      <c r="H73" s="7" t="inlineStr">
+      <c r="H73" s="3" t="inlineStr">
         <is>
           <t>23%</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B74" s="7" t="inlineStr">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Triphasic Thickening Shampoo
 Champô Queda de Cabelo e Cabelo Fino
 500 ml</t>
         </is>
       </c>
-      <c r="D74" s="7" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-thickening-shampoo-8602495.html</t>
         </is>
       </c>
-      <c r="E74" s="7" t="inlineStr"/>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G74" s="7" t="inlineStr">
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
         <is>
           <t>8602495</t>
         </is>
       </c>
-      <c r="H74" s="7" t="inlineStr">
+      <c r="H74" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -17462,40 +17462,40 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B76" s="7" t="inlineStr">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C76" s="7" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>Volumea Volumizing Foam
 Espuma Volumizadora Cabelo Fino sem Volume
 200 ml</t>
         </is>
       </c>
-      <c r="D76" s="7" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/volumea-volumizing-foam-5520281.html</t>
         </is>
       </c>
-      <c r="E76" s="7" t="inlineStr"/>
-      <c r="F76" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G76" s="7" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr"/>
+      <c r="F76" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
         <is>
           <t>5520281</t>
         </is>
       </c>
-      <c r="H76" s="7" t="inlineStr">
+      <c r="H76" s="5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -17611,40 +17611,40 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Biology AC Compensating Cream Ultra-Soothing
 Creme Ultracalmante Tratamento de Acne
 40 ml</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/biology-ac-compensating-cream-ultra-soothing-7756129.html</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>7756129</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -17931,80 +17931,80 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Cutalgan Sting Overheating Roll-on
 Roll-on Refresca Ultra Calmante Pele Irritada
 10 ml</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cutalgan-sting-overheating-roll-on-8124492.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>8124492</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Cytelium Drying Lotion Soothing
 Loção Secante Suavizante Pele Irritada
 100 ml</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/cytelium-drying-lotion-soothing-3691921.html</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>3691921</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18097,43 +18097,43 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>7434584</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18312,83 +18312,83 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Epitheliale Ultra Repair Cream SPF50+
 Creme Protetor Solar Reparador</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/epitheliale-ultra-repair-cream-spf50-412214.html</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>40 ml</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>8478836</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Epitheliale Ultra Repair Massage Gel-Oil HA+
 Gel-óleo Massagem Estrias Ácido Hialurónico
 100 ml</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/epitheliale-ultra-repair-massage-gel-oil-ha-6854488.html</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr"/>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>6854488</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -18515,43 +18515,43 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Exomega Allergo Emollient Balm
 Bálsamo Nutritivo Pele Atópica Alérgica</t>
         </is>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-allergo-emollient-balm-452820.html</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>40 ml</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>7631532</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -18727,43 +18727,43 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>500 ml</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>6587176</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -18813,43 +18813,43 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>8605683</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -20040,40 +20040,40 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Ultra-rich Shower Gel 3in1
 Gel Duche Nutritivo e Calmante Pele Seca
 750 ml</t>
         </is>
       </c>
-      <c r="D61" s="7" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/ultra-rich-shower-gel-3in1-6037067.html</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr"/>
-      <c r="F61" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>6037067</t>
         </is>
       </c>
-      <c r="H61" s="7" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -22100,40 +22100,40 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C50" s="7" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Escova Dentes Próteses Dentárias
 1 un</t>
         </is>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/escova-dentes-proteses-dentarias-4907334.html</t>
         </is>
       </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>4907334</t>
         </is>
       </c>
-      <c r="H50" s="7" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -24716,43 +24716,43 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Dexeryl</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Cleansing Oil Lipid-Replenishing, Soothing
 Óleo de Duche Corpo Pele Seca e Atópica</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cleansing-oil-lipid-replenishing-soothing-443916.html</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>8691147</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -25297,38 +25297,38 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Dermalibour+ Repairing CICA-Cream
 Creme Reparador Purificante Pele Irritada</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>7434584</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/dermalibour-repairing-cica-cream-452821.html</t>
         </is>
@@ -25449,38 +25449,38 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Epitheliale Ultra Repair Cream SPF50+
 Creme Protetor Solar Reparador</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>40 ml</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>8478836</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/epitheliale-ultra-repair-cream-spf50-412214.html</t>
         </is>
@@ -25525,38 +25525,38 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Exomega Allergo Emollient Balm
 Bálsamo Nutritivo Pele Atópica Alérgica</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>40 ml</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>7631532</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-allergo-emollient-balm-452820.html</t>
         </is>
@@ -25639,38 +25639,38 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>8605683</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
@@ -25715,38 +25715,38 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>500 ml</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>6587176</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
@@ -26700,38 +26700,38 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>Dexeryl</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>Cleansing Oil Lipid-Replenishing, Soothing
 Óleo de Duche Corpo Pele Seca e Atópica</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>8691147</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
       </c>
-      <c r="G42" s="7" t="inlineStr">
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cleansing-oil-lipid-replenishing-soothing-443916.html</t>
         </is>
@@ -27308,38 +27308,38 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B58" s="7" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Shampoo
 Champô Camomila Reflexos Dourado Cabelo Loiro</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D58" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>3000697</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
+      <c r="F58" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="G58" s="7" t="inlineStr">
+      <c r="G58" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-shampoo-343981.html</t>
         </is>
@@ -27574,38 +27574,38 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="7" t="inlineStr">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B65" s="7" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>Manga Nourishing Conditioner
 Condicionador Manga Nutritivo Cabelo Seco</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D65" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>6128332</t>
         </is>
       </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G65" s="7" t="inlineStr">
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/manga-nourishing-conditioner-343975.html</t>
         </is>
@@ -27840,38 +27840,38 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>Nettle Oil Control Shampoo
 Champô Ortiga BIO Purifica Cabelo Oleoso</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E72" s="7" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>3688262</t>
         </is>
       </c>
-      <c r="F72" s="7" t="inlineStr">
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="G72" s="7" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/nettle-oil-control-shampoo-343980.html</t>
         </is>
@@ -28106,38 +28106,38 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="7" t="inlineStr">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B79" s="7" t="inlineStr">
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>Oat&amp;Ceramide Ultra-Gentle Dry Shampoo Dark
 Champô Seco Aveia Ultra-Suave Cabelo Castanho</t>
         </is>
       </c>
-      <c r="C79" s="7" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D79" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
         <is>
           <t>7831154</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="inlineStr">
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/oatandceramide-ultra-gentle-dry-shampoo-dark-341982.html</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-03-17 15:28 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_17_03_2026.xlsx
+++ b/logs/Consolidado_17_03_2026.xlsx
@@ -676,10 +676,10 @@
         <v>79</v>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
         <v>2</v>
@@ -11004,43 +11004,43 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Shampoo
 Champô Camomila Reflexos Dourado Cabelo Loiro</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-shampoo-343981.html</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>3000697</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -27308,38 +27308,38 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>Chamomile Brightening Blond Hair Shampoo
 Champô Camomila Reflexos Dourado Cabelo Loiro</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
         <is>
           <t>3000697</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F58" s="7" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="G58" s="3" t="inlineStr">
+      <c r="G58" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/chamomile-brightening-blond-hair-shampoo-343981.html</t>
         </is>

</xml_diff>

<commit_message>
chore: run 2026-03-17 16:41 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_17_03_2026.xlsx
+++ b/logs/Consolidado_17_03_2026.xlsx
@@ -695,10 +695,10 @@
         <v>71</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
@@ -8542,12 +8542,12 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>4289378</t>
+          <t>5732892</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -8585,12 +8585,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>5732892</t>
+          <t>4289378</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>35%</t>
         </is>
       </c>
     </row>
@@ -15888,40 +15888,40 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Okara Blond Brightening Spray Blond Hair
 Spray Cabelo Iluminador Louro Natural ou Pintado
 150 ml</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/okara-blond-brightening-spray-blond-hair-6761000.html</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr"/>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>6761000</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -16888,88 +16888,80 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>Triphasic Active Grow Shampoo
 Champô Crescimento do Cabelo</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-active-grow-shampoo-427541.html</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E62" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>8557861</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr">
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr"/>
+      <c r="H62" s="7" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>17/03/2026</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>Triphasic Active Grow Shampoo
 Champô Crescimento do Cabelo</t>
         </is>
       </c>
-      <c r="D63" s="5" t="inlineStr">
+      <c r="D63" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-active-grow-shampoo-427541.html</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
+      <c r="E63" s="7" t="inlineStr">
         <is>
           <t>500 ml</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G63" s="5" t="inlineStr">
-        <is>
-          <t>8557868</t>
-        </is>
-      </c>
-      <c r="H63" s="5" t="inlineStr">
-        <is>
-          <t>20%</t>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr"/>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -27025,12 +27017,12 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>5732892</t>
+          <t>4289378</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -27063,12 +27055,12 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>4289378</t>
+          <t>5732892</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -28834,76 +28826,68 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="5" t="inlineStr">
+      <c r="A98" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B98" s="5" t="inlineStr">
+      <c r="B98" s="7" t="inlineStr">
         <is>
           <t>Triphasic Active Grow Shampoo
 Champô Crescimento do Cabelo</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
+      <c r="C98" s="7" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E98" s="5" t="inlineStr">
-        <is>
-          <t>8557861</t>
-        </is>
-      </c>
-      <c r="F98" s="5" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="G98" s="5" t="inlineStr">
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr"/>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-active-grow-shampoo-427541.html</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="5" t="inlineStr">
+      <c r="A99" s="7" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="B99" s="5" t="inlineStr">
+      <c r="B99" s="7" t="inlineStr">
         <is>
           <t>Triphasic Active Grow Shampoo
 Champô Crescimento do Cabelo</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
+      <c r="C99" s="7" t="inlineStr">
         <is>
           <t>500 ml</t>
         </is>
       </c>
-      <c r="D99" s="6" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="E99" s="5" t="inlineStr">
-        <is>
-          <t>8557868</t>
-        </is>
-      </c>
-      <c r="F99" s="5" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="G99" s="5" t="inlineStr">
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr"/>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-active-grow-shampoo-427541.html</t>
         </is>

</xml_diff>